<commit_message>
Complete Japan MVP data and scholarship pipeline
</commit_message>
<xml_diff>
--- a/data/sample/06_full_dataset.xlsx
+++ b/data/sample/06_full_dataset.xlsx
@@ -671,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P51"/>
+  <dimension ref="A1:P55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="11" bestFit="1" customWidth="1" style="1" min="1" max="1"/>
@@ -2971,6 +2971,174 @@
       </c>
       <c r="O51" s="3" t="n"/>
       <c r="P51" s="1" t="inlineStr">
+        <is>
+          <t>Pending Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>uni_jp_013</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Ritsumeikan Asia Pacific University</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Beppu</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>https://en.apu.ac.jp/home/</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>https://en.apu.ac.jp/home/</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Pending Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>uni_jp_014</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Soka University</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Hachioji</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>https://www.soka.ac.jp/en/</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>https://www.soka.ac.jp/en/</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Pending Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>uni_jp_015</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Akita University</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Akita</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>https://www.akita-u.ac.jp/eng/</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>https://www.akita-u.ac.jp/eng/</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Pending Verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>uni_jp_016</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>The Graduate University for Advanced Studies, SOKENDAI</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Hayama</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>https://www.soken.ac.jp/en/</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>https://www.soken.ac.jp/en/</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="P55" t="inlineStr">
         <is>
           <t>Pending Verification</t>
         </is>
@@ -5719,7 +5887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
+  <dimension ref="A1:AF13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="14.08984375" customWidth="1" style="12" min="1" max="1"/>
@@ -6037,6 +6205,908 @@
         </is>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sch_jp_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2027 University Recommended Japanese Government MEXT Scholarship</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>uni_jp_001</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Master, PhD</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>https://www.s.u-tokyo.ac.jp/en/admission/scholarship.html</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>https://www.s.u-tokyo.ac.jp/en/admission/scholarship.html</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>sch_jp_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>MEXT IGP Special Quota</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>uni_jp_007</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Master, PhD</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>https://www.global.hokudai.ac.jp/news/26039/</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>https://www.global.hokudai.ac.jp/news/26039/</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sch_jp_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2027 MEXT Scholarship Special Program</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>uni_jp_007</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Master, PhD</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA5" t="inlineStr">
+        <is>
+          <t>https://www2.sci.hokudai.ac.jp/gs/en/news/5419</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr">
+        <is>
+          <t>https://www2.sci.hokudai.ac.jp/gs/en/news/5419</t>
+        </is>
+      </c>
+      <c r="AC5" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE5" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sch_jp_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MEXT Scholarship for International Graduate Program for Advanced Science IGPAS</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>uni_jp_004</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Master</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA6" t="inlineStr">
+        <is>
+          <t>https://www.sci.tohoku.ac.jp/english/prospective/</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>https://www.sci.tohoku.ac.jp/english/prospective/</t>
+        </is>
+      </c>
+      <c r="AC6" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE6" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>sch_jp_008</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MEXT University Recommendation Special Selection AISIP</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>uni_jp_009</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Master, PhD</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>https://www.sie.tsukuba.ac.jp/eng/exam/applicants/entra/</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>https://www.sie.tsukuba.ac.jp/eng/exam/applicants/entra/</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>sch_jp_010</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>MEXT University Recommendation UR Scholarship</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>uni_jp_013</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Master, PhD</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>https://admissions.apu.ac.jp/graduate/how_to_apply/external_scholarship/u_recommendation/</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>https://admissions.apu.ac.jp/graduate/how_to_apply/external_scholarship/u_recommendation/</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sch_jp_012</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>MEXT Foreign Student Priority Placement Special Program</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>uni_jp_014</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>https://www.soka.ac.jp/en/green-technology/gt-mext-scholarship/</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>https://www.soka.ac.jp/en/green-technology/gt-mext-scholarship/</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sch_jp_013</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT Scholarship Undergraduate Program</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>uni_jp_015</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>https://www.akita-u.ac.jp/shigen/eng/reason/program.html</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>https://www.akita-u.ac.jp/shigen/eng/reason/program.html</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>sch_jp_017</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>MEXT Scholarship International Multidisciplinary Engineering Graduate Program IME</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>uni_jp_001</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Master, PhD</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z11" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>https://www.ime.t.u-tokyo.ac.jp/Prospectus-2027.html</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>https://www.ime.t.u-tokyo.ac.jp/Prospectus-2027.html</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>sch_jp_019</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>MEXT Scholarship Student SOKENDAI Recommendation PGP AI and Data Science</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>uni_jp_016</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>https://www.soken.ac.jp/en/admission/application_info/ps/file/Phy_ApplicationGuideline-2027pgp.pdf</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>https://www.soken.ac.jp/en/admission/application_info/ps/file/Phy_ApplicationGuideline-2027pgp.pdf</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>sch_jp_020</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>MEXT Scholarship Student SOKENDAI Recommendation Statistical Science Program</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Japanese Government MEXT</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Government</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>country_jp</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>uni_jp_016</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>PhD</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>Fully Funded</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>upcoming</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>https://www.soken.ac.jp/en/admission/application_info/stat/file/Sta_ApplicationGuideline-2027m.pdf</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>https://www.soken.ac.jp/en/admission/application_info/stat/file/Sta_ApplicationGuideline-2027m.pdf</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>2026-08-11T01:15:03</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>verified</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
Complete programme database sync and South Korea integration
</commit_message>
<xml_diff>
--- a/data/sample/06_full_dataset.xlsx
+++ b/data/sample/06_full_dataset.xlsx
@@ -3160,7 +3160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U37"/>
+  <dimension ref="A1:U82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="11.1796875" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5873,6 +5873,3233 @@
       <c r="U37" t="inlineStr">
         <is>
           <t>Partial - Tuition Verified; Language Classification Verified; Duration Verified; Study Mode Normalized; Admission Requirements Reviewed; No Unverified Numeric Cutoffs Stored; Intake/Deadline Reviewed - Complex Schedule Kept Unstated</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>prog_hk_001</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>uni_hk_001</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Computing and Data Science</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>4</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
+        <v>249000</v>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N38" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O38" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q38" s="15" t="n"/>
+      <c r="R38" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hku.hk/programmes/undergraduate-programmes/computing-and-data-science</t>
+        </is>
+      </c>
+      <c r="S38" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T38" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>prog_hk_002</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>uni_hk_001</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Bachelor of Business Administration</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>4</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
+        <v>224000</v>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O39" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q39" s="15" t="n"/>
+      <c r="R39" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hku.hk/programmes/undergraduate-programmes/bachelor-of-business-administration</t>
+        </is>
+      </c>
+      <c r="S39" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T39" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U39" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>prog_hk_003</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>uni_hk_001</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Bachelor of Science</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>General Science</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F40" t="n">
+        <v>4</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
+        <v>249000</v>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O40" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q40" s="15" t="n"/>
+      <c r="R40" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hku.hk/programmes/undergraduate-programmes/bachelor-of-science</t>
+        </is>
+      </c>
+      <c r="S40" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T40" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>prog_hk_004</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>uni_hk_002</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Computer Science and Engineering</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>4</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
+        <v>214000</v>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q41" s="15" t="n"/>
+      <c r="R41" s="16" t="inlineStr">
+        <is>
+          <t>https://admission.cuhk.edu.hk/programme/bcsen/</t>
+        </is>
+      </c>
+      <c r="S41" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T41" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>prog_hk_005</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>uni_hk_002</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Integrated Bachelor of Business Administration Programme</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F42" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
+        <v>214000</v>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q42" s="15" t="n"/>
+      <c r="R42" s="16" t="inlineStr">
+        <is>
+          <t>https://admission.cuhk.edu.hk/programme/ibbac/</t>
+        </is>
+      </c>
+      <c r="S42" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T42" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>prog_hk_006</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>uni_hk_002</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Data Science and Policy Studies</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>4</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
+        <v>214000</v>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q43" s="15" t="n"/>
+      <c r="R43" s="16" t="inlineStr">
+        <is>
+          <t>https://admission.cuhk.edu.hk/programme/dspsn/</t>
+        </is>
+      </c>
+      <c r="S43" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T43" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>prog_hk_007</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>uni_hk_003</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>BEng in Computer Engineering</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Computer Engineering</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F44" t="n">
+        <v>4</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
+        <v>215000</v>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q44" s="15" t="n"/>
+      <c r="R44" s="16" t="inlineStr">
+        <is>
+          <t>https://join.hkust.edu.hk/our-programs/school-of-engineering/computer-engineering</t>
+        </is>
+      </c>
+      <c r="S44" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T44" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>prog_hk_008</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>uni_hk_003</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>BSc in Biomedical and Health Sciences</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Biomedical &amp; Health Sciences</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>4</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
+        <v>215000</v>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q45" s="15" t="n"/>
+      <c r="R45" s="16" t="inlineStr">
+        <is>
+          <t>https://join.hkust.edu.hk/our-programs/school-of-science/biomedical-and-health-sciences</t>
+        </is>
+      </c>
+      <c r="S45" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T45" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>prog_hk_009</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>uni_hk_003</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>BBA in Economics</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Economics</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F46" t="n">
+        <v>4</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
+        <v>215000</v>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q46" s="15" t="n"/>
+      <c r="R46" s="16" t="inlineStr">
+        <is>
+          <t>https://join.hkust.edu.hk/our-programs/school-of-business-and-management/economics</t>
+        </is>
+      </c>
+      <c r="S46" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T46" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>prog_hk_010</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>uni_hk_004</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) Scheme in Computing and AI</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Intelligent Systems</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>4</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
+        <v>200000</v>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>6</v>
+      </c>
+      <c r="O47" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q47" s="15" t="n"/>
+      <c r="R47" s="16" t="inlineStr">
+        <is>
+          <t>https://www.polyu.edu.hk/study/ug/international/2026/js3868</t>
+        </is>
+      </c>
+      <c r="S47" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T47" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>prog_hk_011</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>uni_hk_004</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) Scheme in Data Science and Artificial Intelligence</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>4</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
+        <v>200000</v>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>6</v>
+      </c>
+      <c r="O48" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q48" s="15" t="n"/>
+      <c r="R48" s="16" t="inlineStr">
+        <is>
+          <t>https://www.polyu.edu.hk/dsai/study/ug/prospective-students/bsc-scheme-in-data-science-and-artificial-intelligence/</t>
+        </is>
+      </c>
+      <c r="S48" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T48" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>prog_hk_012</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>uni_hk_004</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Bachelor's Degree Scheme in Business Administration</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>4</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
+        <v>200000</v>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>6</v>
+      </c>
+      <c r="O49" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q49" s="15" t="n"/>
+      <c r="R49" s="16" t="inlineStr">
+        <is>
+          <t>https://www.polyu.edu.hk/study/ug/international/2026/js3003</t>
+        </is>
+      </c>
+      <c r="S49" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T49" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>prog_hk_013</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>uni_hk_005</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BSc Computer Science</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>4</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O50" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q50" s="15" t="n"/>
+      <c r="R50" s="16" t="inlineStr">
+        <is>
+          <t>https://www.cityu.edu.hk/admo/programmes/bsc-computer-science</t>
+        </is>
+      </c>
+      <c r="S50" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T50" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>prog_hk_014</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>uni_hk_005</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Data Science (Majors: BSc Data Science / BSc Data and Systems Engineering)</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>4</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O51" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q51" s="15" t="n"/>
+      <c r="R51" s="16" t="inlineStr">
+        <is>
+          <t>https://www.cityu.edu.hk/admo/programmes/school-data-science-options-bsc-data-science-bsc-data-and-systems-engineering</t>
+        </is>
+      </c>
+      <c r="S51" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T51" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>prog_hk_015</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>uni_hk_005</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>BBA Global Business</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>4</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="O52" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q52" s="15" t="n"/>
+      <c r="R52" s="16" t="inlineStr">
+        <is>
+          <t>https://www.cityu.edu.hk/admo/programmes/bba-global-business</t>
+        </is>
+      </c>
+      <c r="S52" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T52" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>prog_hk_016</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>uni_hk_006</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Hons) in Business Computing and Data Analytics</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Business Analytics &amp; Information Systems</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>4</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>6</v>
+      </c>
+      <c r="O53" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q53" s="15" t="n"/>
+      <c r="R53" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hkbu.edu.hk/programmes/faculty-of-science/bachelor-of-science-hons-in-business-computing-and-data-analytics-year1.html</t>
+        </is>
+      </c>
+      <c r="S53" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T53" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>prog_hk_017</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>uni_hk_006</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Bachelor of Business Administration (Hons)</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>6</v>
+      </c>
+      <c r="O54" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q54" s="15" t="n"/>
+      <c r="R54" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hkbu.edu.hk/programmes/school-of-business/bachelor-of-business-administration-hons-year1.html</t>
+        </is>
+      </c>
+      <c r="S54" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T54" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>prog_hk_018</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>uni_hk_006</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Bachelor of Communication (Hons) (Journalism and Digital Media / Public Relations and Advertising)</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Communication &amp; Media</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>4</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>English</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>6</v>
+      </c>
+      <c r="O55" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q55" s="15" t="n"/>
+      <c r="R55" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hkbu.edu.hk/programmes/school-of-communication/bachelor-of-communication-hons-journalism-and-digital-media-public-relations-and-advertising-year1.html</t>
+        </is>
+      </c>
+      <c r="S55" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T55" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>prog_hk_019</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>uni_hk_007</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Data Science</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>4</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q56" s="15" t="n"/>
+      <c r="R56" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ln.edu.hk/admissions/ug/programme/jupas-applicants/data-science</t>
+        </is>
+      </c>
+      <c r="S56" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T56" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>prog_hk_020</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>uni_hk_007</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Bachelor of Social Sciences (Honours) - Government and International Affairs</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>International Relations &amp; Public Policy</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>4</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q57" s="15" t="n"/>
+      <c r="R57" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ln.edu.hk/admissions/ug/programme/jupas-applicants/government-and-international-affairs</t>
+        </is>
+      </c>
+      <c r="S57" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T57" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>prog_hk_021</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>uni_hk_007</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Bachelor of Social Sciences (Honours) - Social Data Science</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>4</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q58" s="15" t="n"/>
+      <c r="R58" s="16" t="inlineStr">
+        <is>
+          <t>https://www.ln.edu.hk/admissions/ug/programme/jupas-applicants/social-data-science</t>
+        </is>
+      </c>
+      <c r="S58" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T58" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>prog_hk_022</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>uni_hk_008</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Artificial Intelligence and Educational Technology</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Intelligent Systems</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>4</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
+        <v>180000</v>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q59" s="15" t="n"/>
+      <c r="R59" s="16" t="inlineStr">
+        <is>
+          <t>https://www.apply.eduhk.hk/ug/programmes/aiet</t>
+        </is>
+      </c>
+      <c r="S59" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T59" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>prog_hk_023</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>uni_hk_008</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Bachelor of Arts (Honours) in English Studies and Digital Communication</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Communication &amp; Media</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>4</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
+        <v>180000</v>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q60" s="15" t="n"/>
+      <c r="R60" s="16" t="inlineStr">
+        <is>
+          <t>https://www.apply.eduhk.hk/ug/programmes/esdc/</t>
+        </is>
+      </c>
+      <c r="S60" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T60" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>prog_hk_024</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>uni_hk_008</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Bachelor of Social Sciences (Honours) in Psychology</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>4</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
+        <v>180000</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q61" s="15" t="n"/>
+      <c r="R61" s="16" t="inlineStr">
+        <is>
+          <t>https://www.apply.eduhk.hk/ug/programmes/psy</t>
+        </is>
+      </c>
+      <c r="S61" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T61" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>prog_hk_025</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>uni_hk_009</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Bachelor of Science with Honours in Computing</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>4</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>6</v>
+      </c>
+      <c r="O62" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q62" s="15" t="n"/>
+      <c r="R62" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hkmu.edu.hk/ug/st/bachelor-of-science-with-honours-in-computing/</t>
+        </is>
+      </c>
+      <c r="S62" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T62" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>prog_hk_026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>uni_hk_009</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Bachelor of Business Administration with Honours in Business Management</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>4</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>6</v>
+      </c>
+      <c r="O63" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q63" s="15" t="n"/>
+      <c r="R63" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hkmu.edu.hk/ug/ba/business-management/</t>
+        </is>
+      </c>
+      <c r="S63" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T63" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>prog_hk_027</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>uni_hk_009</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Bachelor of Business Administration with Honours in Finance and Financial Technology</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Finance &amp; Financial Technology</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>4</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>6</v>
+      </c>
+      <c r="O64" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q64" s="15" t="n"/>
+      <c r="R64" s="16" t="inlineStr">
+        <is>
+          <t>https://admissions.hkmu.edu.hk/ug/ba/finance-and-financial-technology/</t>
+        </is>
+      </c>
+      <c r="S64" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T64" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>prog_hk_028</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>uni_hk_010</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Bachelor of Science with Honours in Applied Data Science</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>4</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
+        <v>125675</v>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O65" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q65" s="15" t="n"/>
+      <c r="R65" s="16" t="inlineStr">
+        <is>
+          <t>https://adsci.hksyu.edu/programme/BSc-ADS/programme-overview</t>
+        </is>
+      </c>
+      <c r="S65" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T65" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>prog_hk_029</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>uni_hk_010</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Bachelor of Commerce (Honours) in Financial Technology</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Finance &amp; Financial Technology</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>4</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
+        <v>110089</v>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O66" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q66" s="15" t="n"/>
+      <c r="R66" s="16" t="inlineStr">
+        <is>
+          <t>https://ef.hksyu.edu/Programmes/BCom-in-FinTech</t>
+        </is>
+      </c>
+      <c r="S66" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T66" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>prog_hk_030</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>uni_hk_010</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Bachelor of Social Sciences (Honours) in Psychology</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>4</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
+        <v>110089</v>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O67" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q67" s="15" t="n"/>
+      <c r="R67" s="16" t="inlineStr">
+        <is>
+          <t>https://counpsy.hksyu.edu/</t>
+        </is>
+      </c>
+      <c r="S67" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T67" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>prog_hk_031</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>uni_hk_011</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Applied Computing</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>4</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
+        <v>153820</v>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O68" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q68" s="15" t="n"/>
+      <c r="R68" s="16" t="inlineStr">
+        <is>
+          <t>https://admission.hsu.edu.hk/undergraduate-admissions/year-1-entry/hkdse-sssdp/admission-policy/bachelor-of-science-hons-in-applied-computing-jssh03/</t>
+        </is>
+      </c>
+      <c r="S68" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T68" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>prog_hk_032</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>uni_hk_011</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Data Science and Business Intelligence</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Data Science</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
+        <v>153820</v>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O69" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q69" s="15" t="n"/>
+      <c r="R69" s="16" t="inlineStr">
+        <is>
+          <t>https://msi.hsu.edu.hk/en/dsbi/programme-information/</t>
+        </is>
+      </c>
+      <c r="S69" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T69" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>prog_hk_033</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>uni_hk_011</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Business Analytics and Information Management</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Business Analytics &amp; Information Systems</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
+        <v>153820</v>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O70" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q70" s="15" t="n"/>
+      <c r="R70" s="16" t="inlineStr">
+        <is>
+          <t>https://scm.hsu.edu.hk/baim-msim-programme-overview/</t>
+        </is>
+      </c>
+      <c r="S70" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T70" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>prog_hk_034</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>uni_hk_012</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Hons) in Computer Science</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Computer Science</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>4</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q71" s="15" t="n"/>
+      <c r="R71" s="16" t="inlineStr">
+        <is>
+          <t>https://cs.chuhai.edu.hk/home/?lang=en</t>
+        </is>
+      </c>
+      <c r="S71" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T71" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>prog_hk_035</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>uni_hk_012</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Bachelor of Business Administration (Hons) in Finance and Information Management</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Finance &amp; Financial Technology</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>4</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
+        <v>104750</v>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q72" s="15" t="n"/>
+      <c r="R72" s="16" t="inlineStr">
+        <is>
+          <t>https://fne.chuhai.edu.hk/?page_id=142</t>
+        </is>
+      </c>
+      <c r="S72" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T72" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>prog_hk_036</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>uni_hk_012</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Bachelor of Arts (Hons) in Communication and Digital Media</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Communication &amp; Media</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>4</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
+        <v>104750</v>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q73" s="15" t="n"/>
+      <c r="R73" s="16" t="inlineStr">
+        <is>
+          <t>https://jcm.chuhai.edu.hk/bachelor-of-arts-hons-in-communication-and-digital-media/</t>
+        </is>
+      </c>
+      <c r="S73" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T73" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>prog_hk_037</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>uni_hk_013</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Bachelor of Business Administration (Honours)</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Business &amp; Management</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>4</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
+        <v>100170</v>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q74" s="15" t="n"/>
+      <c r="R74" s="16" t="inlineStr">
+        <is>
+          <t>https://www.sfu.edu.hk/en/admission/programmes-by-qflevel/bachelor-s-degree-programmes/bachelor-of-business-administration-honours/introduction/index.html</t>
+        </is>
+      </c>
+      <c r="S74" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T74" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>prog_hk_038</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>uni_hk_013</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Bachelor of Arts (Honours) in Translation Technology</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Languages &amp; Translation</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>4</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
+        <v>100170</v>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q75" s="15" t="n"/>
+      <c r="R75" s="16" t="inlineStr">
+        <is>
+          <t>https://www.sfu.edu.hk/en/programmes/bachelor-s-degree-programmes/bachelor-of-arts-honours-in-translation-technology/introduction/index.html</t>
+        </is>
+      </c>
+      <c r="S75" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T75" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>prog_hk_039</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>uni_hk_013</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Artificial Intelligence and Multimedia Technology</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Artificial Intelligence &amp; Intelligent Systems</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>4</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
+        <v>106670</v>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N76" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q76" s="15" t="n"/>
+      <c r="R76" s="16" t="inlineStr">
+        <is>
+          <t>https://www.sfu.edu.hk/en/admission/programmes-by-qflevel/bachelor-s-degree-programmes/bachelor-of-science-honours-in-artificial-intelligence-and-multimedia-technology-/introduction/index.html</t>
+        </is>
+      </c>
+      <c r="S76" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T76" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>prog_hk_040</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>uni_hk_014</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Multimedia Technology and Innovation</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Media &amp; Design</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>4</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N77" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O77" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q77" s="15" t="n"/>
+      <c r="R77" s="16" t="inlineStr">
+        <is>
+          <t>https://thei.edu.hk/departments/department-of-digital-innovation-and-technology/bachelor-of-science-honours-multimedia-technology-and-innovation/</t>
+        </is>
+      </c>
+      <c r="S77" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T77" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>prog_hk_041</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>uni_hk_014</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Information and Communications Technology</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Information Science &amp; Informatics</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>4</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N78" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O78" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q78" s="15" t="n"/>
+      <c r="R78" s="16" t="inlineStr">
+        <is>
+          <t>https://thei.edu.hk/departments/department-of-digital-innovation-and-technology/bachelor-of-science-honours-information-and-communications-technology/</t>
+        </is>
+      </c>
+      <c r="S78" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T78" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>prog_hk_042</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>uni_hk_014</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bachelor of Arts (Honours) in Fashion Design</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Fashion &amp; Design</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>4</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="N79" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="O79" t="n">
+        <v>79</v>
+      </c>
+      <c r="Q79" s="15" t="n"/>
+      <c r="R79" s="16" t="inlineStr">
+        <is>
+          <t>https://thei.edu.hk/departments/department-of-design-and-architecture/bachelor-of-arts-honours-fashion-design/</t>
+        </is>
+      </c>
+      <c r="S79" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T79" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>prog_hk_043</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>uni_hk_015</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Bachelor of Social Science (Honours) in Applied Psychology</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Psychology</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>4</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
+        <v>84750</v>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N80" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q80" s="15" t="n"/>
+      <c r="R80" s="16" t="inlineStr">
+        <is>
+          <t>https://www.twc.edu.hk/en/Programmes/bssap/admission_requirement</t>
+        </is>
+      </c>
+      <c r="S80" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T80" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>prog_hk_044</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>uni_hk_015</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Bachelor of Management (Honours) in Social and Business Sustainability</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Sustainability &amp; Social Sciences</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>4</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
+        <v>86170</v>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N81" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q81" s="15" t="n"/>
+      <c r="R81" s="16" t="inlineStr">
+        <is>
+          <t>https://www.twc.edu.hk/en/Programmes/bmgtsbs/admission_requirement</t>
+        </is>
+      </c>
+      <c r="S81" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T81" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>current</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>prog_hk_045</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>uni_hk_015</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Bachelor of Science (Honours) in Biomedical Science</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Biomedical &amp; Health Sciences</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Bachelor</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>4</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>Full-time</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>English Available</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
+        <v>122850</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>HKD</t>
+        </is>
+      </c>
+      <c r="K82" t="inlineStr">
+        <is>
+          <t>Annual</t>
+        </is>
+      </c>
+      <c r="N82" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="Q82" s="15" t="n"/>
+      <c r="R82" s="16" t="inlineStr">
+        <is>
+          <t>https://www.twc.edu.hk/en/Programmes/bsbms</t>
+        </is>
+      </c>
+      <c r="S82" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="T82" s="15" t="n">
+        <v>46255</v>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>current</t>
         </is>
       </c>
     </row>

</xml_diff>